<commit_message>
feat(templates): save and align user replaced Sales template
</commit_message>
<xml_diff>
--- a/app/templates/informes/Sales/1- Info N° 001-26 SU13 Sales-1 Ult.xlsx
+++ b/app/templates/informes/Sales/1- Info N° 001-26 SU13 Sales-1 Ult.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="5" rupBuild="25128"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="5" rupBuild="27928"/>
   <workbookPr codeName="ThisWorkbook"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="G:\Mi unidad\3.0 Formatos e informes\2026\1.0 Informe de ensayo\1.1 Informe Suelo\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Lenovo\Documents\crmnew\api-geofal-crm\app\templates\informes\Sales\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E57CDA9B-30CE-42FC-B17A-E054F5884125}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{BEC0F210-575F-4C70-9503-BB879A54E8D2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" tabRatio="723" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" tabRatio="723" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="FORMATO" sheetId="95" r:id="rId1"/>
@@ -2069,6 +2069,108 @@
       <alignment horizontal="left" vertical="center"/>
       <protection hidden="1"/>
     </xf>
+    <xf numFmtId="0" fontId="17" fillId="3" borderId="0" xfId="3" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="0" borderId="0" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="2" borderId="29" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center"/>
+      <protection hidden="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="2" borderId="30" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center"/>
+      <protection hidden="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="2" borderId="30" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="2" borderId="29" xfId="4" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="3" borderId="10" xfId="4" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="26" fillId="2" borderId="29" xfId="4" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="32" fillId="3" borderId="10" xfId="3" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="0" borderId="29" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center"/>
+      <protection hidden="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center"/>
+      <protection hidden="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="0" borderId="30" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center"/>
+      <protection hidden="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="3" borderId="4" xfId="4" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="3" borderId="3" xfId="4" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="3" borderId="5" xfId="4" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="3" borderId="8" xfId="4" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="3" borderId="2" xfId="4" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="3" borderId="9" xfId="4" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="17" fillId="0" borderId="29" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center"/>
+      <protection hidden="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="17" fillId="0" borderId="30" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center"/>
+      <protection hidden="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+      <protection hidden="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+      <protection hidden="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+      <protection hidden="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+      <protection hidden="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+      <protection hidden="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+      <protection hidden="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="32" fillId="3" borderId="0" xfId="3" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="167" fontId="13" fillId="2" borderId="10" xfId="0" quotePrefix="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="167" fontId="13" fillId="2" borderId="30" xfId="0" quotePrefix="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="2" borderId="30" xfId="4" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="26" fillId="3" borderId="29" xfId="3" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
@@ -2091,106 +2193,42 @@
     <xf numFmtId="0" fontId="31" fillId="0" borderId="30" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="13" fillId="2" borderId="29" xfId="4" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="3" borderId="10" xfId="4" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+    <xf numFmtId="0" fontId="13" fillId="0" borderId="0" xfId="5" quotePrefix="1" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="178" fontId="21" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="17" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
-      <protection hidden="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="23" xfId="4" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
-      <protection hidden="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="17" xfId="4" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
-      <protection hidden="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="29" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
-      <protection hidden="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
-      <protection hidden="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="30" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
-      <protection hidden="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="32" fillId="3" borderId="0" xfId="3" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="13" fillId="0" borderId="29" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center"/>
-      <protection hidden="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="13" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center"/>
-      <protection hidden="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="13" fillId="0" borderId="30" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center"/>
-      <protection hidden="1"/>
-    </xf>
-    <xf numFmtId="167" fontId="13" fillId="2" borderId="10" xfId="0" quotePrefix="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="167" fontId="13" fillId="2" borderId="30" xfId="0" quotePrefix="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="13" fillId="2" borderId="30" xfId="4" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="26" fillId="2" borderId="29" xfId="4" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="32" fillId="3" borderId="10" xfId="3" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="13" fillId="3" borderId="4" xfId="4" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    </xf>
+    <xf numFmtId="0" fontId="27" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="left" vertical="center"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="27" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1" applyProtection="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="13" fillId="3" borderId="3" xfId="4" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="13" fillId="3" borderId="5" xfId="4" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="13" fillId="3" borderId="8" xfId="4" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="13" fillId="3" borderId="2" xfId="4" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="13" fillId="3" borderId="9" xfId="4" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="17" fillId="0" borderId="29" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center"/>
-      <protection hidden="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="17" fillId="0" borderId="30" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center"/>
-      <protection hidden="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="17" fillId="3" borderId="0" xfId="3" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="13" fillId="0" borderId="0" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="13" fillId="2" borderId="29" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center"/>
-      <protection hidden="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="13" fillId="2" borderId="30" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center"/>
-      <protection hidden="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="2" borderId="30" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center"/>
       <protection locked="0"/>
     </xf>
     <xf numFmtId="0" fontId="7" fillId="0" borderId="21" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
@@ -2254,44 +2292,6 @@
     </xf>
     <xf numFmtId="0" fontId="9" fillId="0" borderId="0" xfId="3" applyFont="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="27" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="13" fillId="0" borderId="0" xfId="5" quotePrefix="1" applyFont="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="21" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="178" fontId="21" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="17" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="23" xfId="4" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="17" xfId="4" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="29" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="30" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="27" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="left" vertical="center"/>
-      <protection locked="0"/>
     </xf>
     <xf numFmtId="1" fontId="9" fillId="0" borderId="23" xfId="4" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -3831,32 +3831,32 @@
       <c r="M5" s="272"/>
     </row>
     <row r="6" spans="1:13" ht="15.9" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A6" s="286" t="s">
+      <c r="A6" s="316" t="s">
         <v>17</v>
       </c>
-      <c r="B6" s="286"/>
-      <c r="C6" s="286"/>
-      <c r="D6" s="286"/>
-      <c r="E6" s="286"/>
-      <c r="F6" s="286"/>
-      <c r="G6" s="286"/>
-      <c r="H6" s="286"/>
-      <c r="I6" s="286"/>
+      <c r="B6" s="316"/>
+      <c r="C6" s="316"/>
+      <c r="D6" s="316"/>
+      <c r="E6" s="316"/>
+      <c r="F6" s="316"/>
+      <c r="G6" s="316"/>
+      <c r="H6" s="316"/>
+      <c r="I6" s="316"/>
       <c r="L6" s="273"/>
       <c r="M6" s="274"/>
     </row>
     <row r="7" spans="1:13" ht="15.9" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A7" s="287" t="s">
+      <c r="A7" s="317" t="s">
         <v>87</v>
       </c>
-      <c r="B7" s="287"/>
-      <c r="C7" s="287"/>
-      <c r="D7" s="287"/>
-      <c r="E7" s="287"/>
-      <c r="F7" s="287"/>
-      <c r="G7" s="287"/>
-      <c r="H7" s="287"/>
-      <c r="I7" s="287"/>
+      <c r="B7" s="317"/>
+      <c r="C7" s="317"/>
+      <c r="D7" s="317"/>
+      <c r="E7" s="317"/>
+      <c r="F7" s="317"/>
+      <c r="G7" s="317"/>
+      <c r="H7" s="317"/>
+      <c r="I7" s="317"/>
       <c r="L7" s="270" t="s">
         <v>86</v>
       </c>
@@ -3872,21 +3872,21 @@
       <c r="M8" s="275"/>
     </row>
     <row r="9" spans="1:13" ht="15.9" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B9" s="288" t="s">
+      <c r="B9" s="318" t="s">
         <v>88</v>
       </c>
-      <c r="C9" s="288"/>
+      <c r="C9" s="318"/>
       <c r="D9" s="206" t="s">
         <v>16</v>
       </c>
-      <c r="E9" s="289" t="s">
+      <c r="E9" s="319" t="s">
         <v>89</v>
       </c>
-      <c r="F9" s="290"/>
-      <c r="G9" s="289" t="s">
+      <c r="F9" s="320"/>
+      <c r="G9" s="319" t="s">
         <v>90</v>
       </c>
-      <c r="H9" s="290"/>
+      <c r="H9" s="320"/>
       <c r="I9"/>
       <c r="J9"/>
       <c r="K9" s="207"/>
@@ -3897,13 +3897,13 @@
     </row>
     <row r="10" spans="1:13" ht="15.9" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A10" s="208"/>
-      <c r="B10" s="284"/>
-      <c r="C10" s="285"/>
+      <c r="B10" s="314"/>
+      <c r="C10" s="315"/>
       <c r="D10" s="209"/>
-      <c r="E10" s="284"/>
-      <c r="F10" s="285"/>
-      <c r="G10" s="284"/>
-      <c r="H10" s="285"/>
+      <c r="E10" s="314"/>
+      <c r="F10" s="315"/>
+      <c r="G10" s="314"/>
+      <c r="H10" s="315"/>
       <c r="I10" s="210"/>
       <c r="J10" s="207"/>
       <c r="K10" s="207"/>
@@ -3928,17 +3928,17 @@
       <c r="M11" s="274"/>
     </row>
     <row r="12" spans="1:13" ht="24.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A12" s="293" t="s">
+      <c r="A12" s="304" t="s">
         <v>91</v>
       </c>
-      <c r="B12" s="294"/>
-      <c r="C12" s="294"/>
-      <c r="D12" s="294"/>
-      <c r="E12" s="294"/>
-      <c r="F12" s="294"/>
-      <c r="G12" s="294"/>
-      <c r="H12" s="294"/>
-      <c r="I12" s="295"/>
+      <c r="B12" s="305"/>
+      <c r="C12" s="305"/>
+      <c r="D12" s="305"/>
+      <c r="E12" s="305"/>
+      <c r="F12" s="305"/>
+      <c r="G12" s="305"/>
+      <c r="H12" s="305"/>
+      <c r="I12" s="306"/>
       <c r="J12" s="207"/>
       <c r="K12" s="207"/>
       <c r="L12" s="270" t="s">
@@ -3947,17 +3947,17 @@
       <c r="M12" s="275"/>
     </row>
     <row r="13" spans="1:13" ht="18" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A13" s="296" t="s">
+      <c r="A13" s="307" t="s">
         <v>23</v>
       </c>
-      <c r="B13" s="297"/>
-      <c r="C13" s="297"/>
-      <c r="D13" s="297"/>
-      <c r="E13" s="297"/>
-      <c r="F13" s="297"/>
-      <c r="G13" s="297"/>
-      <c r="H13" s="297"/>
-      <c r="I13" s="298"/>
+      <c r="B13" s="308"/>
+      <c r="C13" s="308"/>
+      <c r="D13" s="308"/>
+      <c r="E13" s="308"/>
+      <c r="F13" s="308"/>
+      <c r="G13" s="308"/>
+      <c r="H13" s="308"/>
+      <c r="I13" s="309"/>
       <c r="J13" s="207"/>
       <c r="K13" s="207"/>
       <c r="L13" s="270" t="s">
@@ -3981,11 +3981,11 @@
       <c r="M14" s="274"/>
     </row>
     <row r="15" spans="1:13" ht="15.9" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="C15" s="299"/>
-      <c r="D15" s="299"/>
-      <c r="E15" s="299"/>
-      <c r="G15" s="299"/>
-      <c r="H15" s="299"/>
+      <c r="C15" s="310"/>
+      <c r="D15" s="310"/>
+      <c r="E15" s="310"/>
+      <c r="G15" s="310"/>
+      <c r="H15" s="310"/>
       <c r="I15" s="218"/>
       <c r="K15" s="207"/>
       <c r="L15" s="270" t="s">
@@ -4030,17 +4030,17 @@
       <c r="K18" s="207"/>
     </row>
     <row r="19" spans="1:13" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A19" s="300" t="s">
+      <c r="A19" s="293" t="s">
         <v>92</v>
       </c>
-      <c r="B19" s="301"/>
-      <c r="C19" s="301"/>
-      <c r="D19" s="301"/>
-      <c r="E19" s="301"/>
-      <c r="F19" s="301"/>
-      <c r="G19" s="301"/>
-      <c r="H19" s="301"/>
-      <c r="I19" s="302"/>
+      <c r="B19" s="294"/>
+      <c r="C19" s="294"/>
+      <c r="D19" s="294"/>
+      <c r="E19" s="294"/>
+      <c r="F19" s="294"/>
+      <c r="G19" s="294"/>
+      <c r="H19" s="294"/>
+      <c r="I19" s="295"/>
       <c r="K19" s="207"/>
     </row>
     <row r="20" spans="1:13" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
@@ -4077,16 +4077,16 @@
       <c r="B22" s="235" t="s">
         <v>95</v>
       </c>
-      <c r="C22" s="291" t="s">
+      <c r="C22" s="289" t="s">
         <v>24</v>
       </c>
-      <c r="D22" s="303"/>
-      <c r="E22" s="303"/>
+      <c r="D22" s="311"/>
+      <c r="E22" s="311"/>
       <c r="F22" s="231" t="s">
         <v>25</v>
       </c>
-      <c r="G22" s="304"/>
-      <c r="H22" s="304"/>
+      <c r="G22" s="312"/>
+      <c r="H22" s="312"/>
       <c r="I22" s="236"/>
       <c r="J22" s="207"/>
       <c r="K22" s="237"/>
@@ -4096,16 +4096,16 @@
       <c r="B23" s="235" t="s">
         <v>96</v>
       </c>
-      <c r="C23" s="291" t="s">
+      <c r="C23" s="289" t="s">
         <v>26</v>
       </c>
-      <c r="D23" s="292"/>
-      <c r="E23" s="292"/>
+      <c r="D23" s="290"/>
+      <c r="E23" s="290"/>
       <c r="F23" s="231" t="s">
         <v>27</v>
       </c>
-      <c r="G23" s="305"/>
-      <c r="H23" s="305"/>
+      <c r="G23" s="313"/>
+      <c r="H23" s="313"/>
       <c r="I23" s="236"/>
       <c r="J23" s="207"/>
       <c r="K23" s="237"/>
@@ -4115,16 +4115,16 @@
       <c r="B24" s="235" t="s">
         <v>97</v>
       </c>
-      <c r="C24" s="291" t="s">
+      <c r="C24" s="289" t="s">
         <v>28</v>
       </c>
-      <c r="D24" s="292"/>
-      <c r="E24" s="292"/>
+      <c r="D24" s="290"/>
+      <c r="E24" s="290"/>
       <c r="F24" s="231" t="s">
         <v>25</v>
       </c>
-      <c r="G24" s="305"/>
-      <c r="H24" s="305"/>
+      <c r="G24" s="313"/>
+      <c r="H24" s="313"/>
       <c r="I24" s="238"/>
       <c r="J24" s="239"/>
       <c r="K24" s="237"/>
@@ -4134,11 +4134,11 @@
       <c r="B25" s="235" t="s">
         <v>98</v>
       </c>
-      <c r="C25" s="291" t="s">
+      <c r="C25" s="289" t="s">
         <v>29</v>
       </c>
-      <c r="D25" s="292"/>
-      <c r="E25" s="292"/>
+      <c r="D25" s="290"/>
+      <c r="E25" s="290"/>
       <c r="F25" s="231" t="s">
         <v>27</v>
       </c>
@@ -4153,11 +4153,11 @@
       <c r="B26" s="235" t="s">
         <v>99</v>
       </c>
-      <c r="C26" s="291" t="s">
+      <c r="C26" s="289" t="s">
         <v>30</v>
       </c>
-      <c r="D26" s="292"/>
-      <c r="E26" s="292"/>
+      <c r="D26" s="290"/>
+      <c r="E26" s="290"/>
       <c r="F26" s="231" t="s">
         <v>27</v>
       </c>
@@ -4172,11 +4172,11 @@
       <c r="B27" s="235" t="s">
         <v>100</v>
       </c>
-      <c r="C27" s="291" t="s">
+      <c r="C27" s="289" t="s">
         <v>101</v>
       </c>
-      <c r="D27" s="292"/>
-      <c r="E27" s="292"/>
+      <c r="D27" s="290"/>
+      <c r="E27" s="290"/>
       <c r="F27" s="231" t="s">
         <v>27</v>
       </c>
@@ -4191,11 +4191,11 @@
       <c r="B28" s="235" t="s">
         <v>102</v>
       </c>
-      <c r="C28" s="306" t="s">
+      <c r="C28" s="291" t="s">
         <v>103</v>
       </c>
-      <c r="D28" s="307"/>
-      <c r="E28" s="307"/>
+      <c r="D28" s="292"/>
+      <c r="E28" s="292"/>
       <c r="F28" s="241" t="s">
         <v>35</v>
       </c>
@@ -4219,17 +4219,17 @@
       <c r="K29" s="207"/>
     </row>
     <row r="30" spans="1:13" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A30" s="300" t="s">
+      <c r="A30" s="293" t="s">
         <v>104</v>
       </c>
-      <c r="B30" s="301"/>
-      <c r="C30" s="301"/>
-      <c r="D30" s="301"/>
-      <c r="E30" s="301"/>
-      <c r="F30" s="301"/>
-      <c r="G30" s="301"/>
-      <c r="H30" s="301"/>
-      <c r="I30" s="302"/>
+      <c r="B30" s="294"/>
+      <c r="C30" s="294"/>
+      <c r="D30" s="294"/>
+      <c r="E30" s="294"/>
+      <c r="F30" s="294"/>
+      <c r="G30" s="294"/>
+      <c r="H30" s="294"/>
+      <c r="I30" s="295"/>
       <c r="J30" s="207"/>
       <c r="K30" s="207"/>
     </row>
@@ -4345,14 +4345,14 @@
     <row r="38" spans="1:11" ht="18" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A38" s="255"/>
       <c r="B38" s="47"/>
-      <c r="C38" s="308" t="s">
+      <c r="C38" s="296" t="s">
         <v>109</v>
       </c>
-      <c r="D38" s="309"/>
-      <c r="E38" s="309"/>
-      <c r="F38" s="309"/>
-      <c r="G38" s="309"/>
-      <c r="H38" s="310"/>
+      <c r="D38" s="297"/>
+      <c r="E38" s="297"/>
+      <c r="F38" s="297"/>
+      <c r="G38" s="297"/>
+      <c r="H38" s="298"/>
       <c r="I38" s="240"/>
       <c r="J38" s="207"/>
       <c r="K38" s="207"/>
@@ -4360,12 +4360,12 @@
     <row r="39" spans="1:11" ht="18" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A39" s="255"/>
       <c r="B39" s="47"/>
-      <c r="C39" s="311"/>
-      <c r="D39" s="312"/>
-      <c r="E39" s="312"/>
-      <c r="F39" s="312"/>
-      <c r="G39" s="312"/>
-      <c r="H39" s="313"/>
+      <c r="C39" s="299"/>
+      <c r="D39" s="300"/>
+      <c r="E39" s="300"/>
+      <c r="F39" s="300"/>
+      <c r="G39" s="300"/>
+      <c r="H39" s="301"/>
       <c r="I39" s="240"/>
       <c r="J39" s="207"/>
       <c r="K39" s="207"/>
@@ -4399,14 +4399,14 @@
     <row r="42" spans="1:11" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A42" s="262"/>
       <c r="B42" s="262"/>
-      <c r="C42" s="314" t="s">
+      <c r="C42" s="302" t="s">
         <v>110</v>
       </c>
-      <c r="D42" s="315"/>
-      <c r="E42" s="314" t="s">
+      <c r="D42" s="303"/>
+      <c r="E42" s="302" t="s">
         <v>111</v>
       </c>
-      <c r="F42" s="315"/>
+      <c r="F42" s="303"/>
       <c r="G42" s="265"/>
       <c r="H42" s="265"/>
       <c r="I42" s="262"/>
@@ -4416,12 +4416,12 @@
     <row r="43" spans="1:11" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A43" s="262"/>
       <c r="B43" s="262"/>
-      <c r="C43" s="318" t="s">
+      <c r="C43" s="286" t="s">
         <v>112</v>
       </c>
-      <c r="D43" s="319"/>
-      <c r="E43" s="320"/>
-      <c r="F43" s="320"/>
+      <c r="D43" s="287"/>
+      <c r="E43" s="288"/>
+      <c r="F43" s="288"/>
       <c r="G43" s="265"/>
       <c r="H43" s="265"/>
       <c r="I43" s="262"/>
@@ -4431,12 +4431,12 @@
     <row r="44" spans="1:11" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A44" s="262"/>
       <c r="B44" s="262"/>
-      <c r="C44" s="318" t="s">
+      <c r="C44" s="286" t="s">
         <v>113</v>
       </c>
-      <c r="D44" s="319"/>
-      <c r="E44" s="320"/>
-      <c r="F44" s="320"/>
+      <c r="D44" s="287"/>
+      <c r="E44" s="288"/>
+      <c r="F44" s="288"/>
       <c r="G44" s="265"/>
       <c r="H44" s="265"/>
       <c r="I44" s="262"/>
@@ -4446,12 +4446,12 @@
     <row r="45" spans="1:11" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A45" s="262"/>
       <c r="B45" s="262"/>
-      <c r="C45" s="318" t="s">
+      <c r="C45" s="286" t="s">
         <v>114</v>
       </c>
-      <c r="D45" s="319"/>
-      <c r="E45" s="320"/>
-      <c r="F45" s="320"/>
+      <c r="D45" s="287"/>
+      <c r="E45" s="288"/>
+      <c r="F45" s="288"/>
       <c r="G45" s="265"/>
       <c r="H45" s="265"/>
       <c r="I45" s="262"/>
@@ -4531,12 +4531,12 @@
       <c r="K51" s="207"/>
     </row>
     <row r="52" spans="1:11" ht="15.9" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B52" s="316"/>
-      <c r="C52" s="316"/>
-      <c r="D52" s="316"/>
-      <c r="E52" s="316"/>
-      <c r="F52" s="316"/>
-      <c r="G52" s="316"/>
+      <c r="B52" s="284"/>
+      <c r="C52" s="284"/>
+      <c r="D52" s="284"/>
+      <c r="E52" s="284"/>
+      <c r="F52" s="284"/>
+      <c r="G52" s="284"/>
       <c r="H52" s="211"/>
       <c r="I52" s="46"/>
       <c r="J52" s="207"/>
@@ -4575,41 +4575,35 @@
     </row>
     <row r="55" spans="1:11" ht="15.9" customHeight="1" x14ac:dyDescent="0.25"/>
     <row r="56" spans="1:11" ht="30.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A56" s="317" t="s">
+      <c r="A56" s="285" t="s">
         <v>117</v>
       </c>
-      <c r="B56" s="317"/>
-      <c r="C56" s="317"/>
-      <c r="D56" s="317"/>
-      <c r="E56" s="317"/>
-      <c r="F56" s="317"/>
-      <c r="G56" s="317"/>
-      <c r="H56" s="317"/>
-      <c r="I56" s="317"/>
+      <c r="B56" s="285"/>
+      <c r="C56" s="285"/>
+      <c r="D56" s="285"/>
+      <c r="E56" s="285"/>
+      <c r="F56" s="285"/>
+      <c r="G56" s="285"/>
+      <c r="H56" s="285"/>
+      <c r="I56" s="285"/>
     </row>
     <row r="57" spans="1:11" ht="15.9" customHeight="1" x14ac:dyDescent="0.25"/>
     <row r="58" spans="1:11" ht="15.9" customHeight="1" x14ac:dyDescent="0.25"/>
   </sheetData>
+  <sheetProtection sheet="1" objects="1" scenarios="1"/>
   <protectedRanges>
     <protectedRange sqref="C11 C14" name="Rango3_3_1_1_1_1_1_1_1_1"/>
     <protectedRange sqref="C52" name="Rango3_3_1_1_1_1_1_2_1"/>
   </protectedRanges>
   <mergeCells count="36">
-    <mergeCell ref="B52:D52"/>
-    <mergeCell ref="E52:G52"/>
-    <mergeCell ref="A56:I56"/>
-    <mergeCell ref="C43:D43"/>
-    <mergeCell ref="E43:F43"/>
-    <mergeCell ref="C44:D44"/>
-    <mergeCell ref="E44:F44"/>
-    <mergeCell ref="C45:D45"/>
-    <mergeCell ref="E45:F45"/>
-    <mergeCell ref="C27:E27"/>
-    <mergeCell ref="C28:E28"/>
-    <mergeCell ref="A30:I30"/>
-    <mergeCell ref="C38:H39"/>
-    <mergeCell ref="C42:D42"/>
-    <mergeCell ref="E42:F42"/>
+    <mergeCell ref="B10:C10"/>
+    <mergeCell ref="A6:I6"/>
+    <mergeCell ref="A7:I7"/>
+    <mergeCell ref="B9:C9"/>
+    <mergeCell ref="E9:F9"/>
+    <mergeCell ref="G9:H9"/>
+    <mergeCell ref="E10:F10"/>
+    <mergeCell ref="G10:H10"/>
     <mergeCell ref="C26:E26"/>
     <mergeCell ref="A12:I12"/>
     <mergeCell ref="A13:I13"/>
@@ -4623,14 +4617,21 @@
     <mergeCell ref="C24:E24"/>
     <mergeCell ref="G24:H24"/>
     <mergeCell ref="C25:E25"/>
-    <mergeCell ref="B10:C10"/>
-    <mergeCell ref="A6:I6"/>
-    <mergeCell ref="A7:I7"/>
-    <mergeCell ref="B9:C9"/>
-    <mergeCell ref="E9:F9"/>
-    <mergeCell ref="G9:H9"/>
-    <mergeCell ref="E10:F10"/>
-    <mergeCell ref="G10:H10"/>
+    <mergeCell ref="C27:E27"/>
+    <mergeCell ref="C28:E28"/>
+    <mergeCell ref="A30:I30"/>
+    <mergeCell ref="C38:H39"/>
+    <mergeCell ref="C42:D42"/>
+    <mergeCell ref="E42:F42"/>
+    <mergeCell ref="B52:D52"/>
+    <mergeCell ref="E52:G52"/>
+    <mergeCell ref="A56:I56"/>
+    <mergeCell ref="C43:D43"/>
+    <mergeCell ref="E43:F43"/>
+    <mergeCell ref="C44:D44"/>
+    <mergeCell ref="E44:F44"/>
+    <mergeCell ref="C45:D45"/>
+    <mergeCell ref="E45:F45"/>
   </mergeCells>
   <printOptions horizontalCentered="1" verticalCentered="1"/>
   <pageMargins left="0.78740157480314965" right="0.78740157480314965" top="0.78740157480314965" bottom="0.39370078740157483" header="0" footer="0"/>
@@ -4772,38 +4773,38 @@
       <c r="M7" s="15"/>
     </row>
     <row r="8" spans="1:20" ht="15.9" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A8" s="342" t="s">
+      <c r="A8" s="322" t="s">
         <v>17</v>
       </c>
-      <c r="B8" s="342"/>
-      <c r="C8" s="342"/>
-      <c r="D8" s="342"/>
-      <c r="E8" s="342"/>
-      <c r="F8" s="342"/>
-      <c r="G8" s="342"/>
-      <c r="H8" s="342"/>
-      <c r="I8" s="342"/>
-      <c r="J8" s="342"/>
-      <c r="K8" s="342"/>
-      <c r="L8" s="342"/>
-      <c r="M8" s="342"/>
+      <c r="B8" s="322"/>
+      <c r="C8" s="322"/>
+      <c r="D8" s="322"/>
+      <c r="E8" s="322"/>
+      <c r="F8" s="322"/>
+      <c r="G8" s="322"/>
+      <c r="H8" s="322"/>
+      <c r="I8" s="322"/>
+      <c r="J8" s="322"/>
+      <c r="K8" s="322"/>
+      <c r="L8" s="322"/>
+      <c r="M8" s="322"/>
     </row>
     <row r="9" spans="1:20" ht="15.9" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A9" s="343">
+      <c r="A9" s="323">
         <v>1</v>
       </c>
-      <c r="B9" s="343"/>
-      <c r="C9" s="343"/>
-      <c r="D9" s="343"/>
-      <c r="E9" s="343"/>
-      <c r="F9" s="343"/>
-      <c r="G9" s="343"/>
-      <c r="H9" s="343"/>
-      <c r="I9" s="343"/>
-      <c r="J9" s="343"/>
-      <c r="K9" s="343"/>
-      <c r="L9" s="343"/>
-      <c r="M9" s="343"/>
+      <c r="B9" s="323"/>
+      <c r="C9" s="323"/>
+      <c r="D9" s="323"/>
+      <c r="E9" s="323"/>
+      <c r="F9" s="323"/>
+      <c r="G9" s="323"/>
+      <c r="H9" s="323"/>
+      <c r="I9" s="323"/>
+      <c r="J9" s="323"/>
+      <c r="K9" s="323"/>
+      <c r="L9" s="323"/>
+      <c r="M9" s="323"/>
       <c r="R9" s="158"/>
     </row>
     <row r="10" spans="1:20" ht="15.9" customHeight="1" x14ac:dyDescent="0.25">
@@ -4828,17 +4829,17 @@
       <c r="B11" s="17" t="s">
         <v>0</v>
       </c>
-      <c r="C11" s="340">
+      <c r="C11" s="331">
         <f>+FORMATO!M2</f>
         <v>0</v>
       </c>
-      <c r="D11" s="340"/>
-      <c r="E11" s="340"/>
-      <c r="F11" s="340"/>
-      <c r="G11" s="340"/>
-      <c r="H11" s="340"/>
-      <c r="I11" s="340"/>
-      <c r="J11" s="340"/>
+      <c r="D11" s="331"/>
+      <c r="E11" s="331"/>
+      <c r="F11" s="331"/>
+      <c r="G11" s="331"/>
+      <c r="H11" s="331"/>
+      <c r="I11" s="331"/>
+      <c r="J11" s="331"/>
       <c r="K11" s="19" t="s">
         <v>21</v>
       </c>
@@ -4860,17 +4861,17 @@
       <c r="B12" s="17" t="s">
         <v>0</v>
       </c>
-      <c r="C12" s="350">
+      <c r="C12" s="330">
         <f>+FORMATO!M3</f>
         <v>0</v>
       </c>
-      <c r="D12" s="350"/>
-      <c r="E12" s="350"/>
-      <c r="F12" s="350"/>
-      <c r="G12" s="350"/>
-      <c r="H12" s="350"/>
-      <c r="I12" s="350"/>
-      <c r="J12" s="350"/>
+      <c r="D12" s="330"/>
+      <c r="E12" s="330"/>
+      <c r="F12" s="330"/>
+      <c r="G12" s="330"/>
+      <c r="H12" s="330"/>
+      <c r="I12" s="330"/>
+      <c r="J12" s="330"/>
       <c r="K12" s="278" t="s">
         <v>86</v>
       </c>
@@ -4895,17 +4896,17 @@
       <c r="B13" s="17" t="s">
         <v>0</v>
       </c>
-      <c r="C13" s="340">
+      <c r="C13" s="331">
         <f>+FORMATO!M4</f>
         <v>0</v>
       </c>
-      <c r="D13" s="340"/>
-      <c r="E13" s="340"/>
-      <c r="F13" s="340"/>
-      <c r="G13" s="340"/>
-      <c r="H13" s="340"/>
-      <c r="I13" s="340"/>
-      <c r="J13" s="340"/>
+      <c r="D13" s="331"/>
+      <c r="E13" s="331"/>
+      <c r="F13" s="331"/>
+      <c r="G13" s="331"/>
+      <c r="H13" s="331"/>
+      <c r="I13" s="331"/>
+      <c r="J13" s="331"/>
       <c r="K13" s="21" t="s">
         <v>63</v>
       </c>
@@ -4919,8 +4920,8 @@
       <c r="N13" s="111"/>
       <c r="O13" s="111"/>
       <c r="P13" s="111"/>
-      <c r="S13" s="324"/>
-      <c r="T13" s="324"/>
+      <c r="S13" s="335"/>
+      <c r="T13" s="335"/>
     </row>
     <row r="14" spans="1:20" ht="17.399999999999999" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A14" s="68" t="s">
@@ -4929,18 +4930,18 @@
       <c r="B14" s="17" t="s">
         <v>0</v>
       </c>
-      <c r="C14" s="340">
+      <c r="C14" s="331">
         <f>+FORMATO!M5</f>
         <v>0</v>
       </c>
-      <c r="D14" s="340"/>
-      <c r="E14" s="340"/>
-      <c r="F14" s="340"/>
-      <c r="G14" s="340"/>
-      <c r="H14" s="340"/>
-      <c r="I14" s="340"/>
-      <c r="J14" s="340"/>
-      <c r="K14" s="340"/>
+      <c r="D14" s="331"/>
+      <c r="E14" s="331"/>
+      <c r="F14" s="331"/>
+      <c r="G14" s="331"/>
+      <c r="H14" s="331"/>
+      <c r="I14" s="331"/>
+      <c r="J14" s="331"/>
+      <c r="K14" s="331"/>
       <c r="L14" s="17"/>
       <c r="M14" s="62"/>
       <c r="N14" s="111"/>
@@ -4972,21 +4973,21 @@
       <c r="T15" s="160"/>
     </row>
     <row r="16" spans="1:20" ht="30" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A16" s="325" t="s">
+      <c r="A16" s="336" t="s">
         <v>80</v>
       </c>
-      <c r="B16" s="326"/>
-      <c r="C16" s="326"/>
-      <c r="D16" s="326"/>
-      <c r="E16" s="326"/>
-      <c r="F16" s="326"/>
-      <c r="G16" s="326"/>
-      <c r="H16" s="326"/>
-      <c r="I16" s="326"/>
-      <c r="J16" s="326"/>
-      <c r="K16" s="326"/>
-      <c r="L16" s="326"/>
-      <c r="M16" s="327"/>
+      <c r="B16" s="337"/>
+      <c r="C16" s="337"/>
+      <c r="D16" s="337"/>
+      <c r="E16" s="337"/>
+      <c r="F16" s="337"/>
+      <c r="G16" s="337"/>
+      <c r="H16" s="337"/>
+      <c r="I16" s="337"/>
+      <c r="J16" s="337"/>
+      <c r="K16" s="337"/>
+      <c r="L16" s="337"/>
+      <c r="M16" s="338"/>
       <c r="N16" s="111"/>
       <c r="O16" s="111"/>
       <c r="P16" s="111"/>
@@ -4994,21 +4995,21 @@
       <c r="T16" s="160"/>
     </row>
     <row r="17" spans="1:20" ht="18" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A17" s="331" t="s">
+      <c r="A17" s="342" t="s">
         <v>23</v>
       </c>
-      <c r="B17" s="332"/>
-      <c r="C17" s="332"/>
-      <c r="D17" s="332"/>
-      <c r="E17" s="332"/>
-      <c r="F17" s="332"/>
-      <c r="G17" s="332"/>
-      <c r="H17" s="332"/>
-      <c r="I17" s="332"/>
-      <c r="J17" s="332"/>
-      <c r="K17" s="332"/>
-      <c r="L17" s="332"/>
-      <c r="M17" s="333"/>
+      <c r="B17" s="343"/>
+      <c r="C17" s="343"/>
+      <c r="D17" s="343"/>
+      <c r="E17" s="343"/>
+      <c r="F17" s="343"/>
+      <c r="G17" s="343"/>
+      <c r="H17" s="343"/>
+      <c r="I17" s="343"/>
+      <c r="J17" s="343"/>
+      <c r="K17" s="343"/>
+      <c r="L17" s="343"/>
+      <c r="M17" s="344"/>
       <c r="N17" s="111"/>
       <c r="O17" s="111"/>
       <c r="P17" s="111"/>
@@ -5036,33 +5037,33 @@
       <c r="T18" s="160"/>
     </row>
     <row r="19" spans="1:20" ht="15.9" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A19" s="328" t="s">
+      <c r="A19" s="339" t="s">
         <v>20</v>
       </c>
-      <c r="B19" s="329"/>
-      <c r="C19" s="329"/>
-      <c r="D19" s="329"/>
-      <c r="E19" s="329"/>
-      <c r="F19" s="329"/>
-      <c r="G19" s="329"/>
-      <c r="H19" s="329"/>
-      <c r="I19" s="329"/>
-      <c r="J19" s="329"/>
-      <c r="K19" s="329"/>
-      <c r="L19" s="329"/>
-      <c r="M19" s="330"/>
+      <c r="B19" s="340"/>
+      <c r="C19" s="340"/>
+      <c r="D19" s="340"/>
+      <c r="E19" s="340"/>
+      <c r="F19" s="340"/>
+      <c r="G19" s="340"/>
+      <c r="H19" s="340"/>
+      <c r="I19" s="340"/>
+      <c r="J19" s="340"/>
+      <c r="K19" s="340"/>
+      <c r="L19" s="340"/>
+      <c r="M19" s="341"/>
       <c r="O19" s="111"/>
       <c r="P19" s="111"/>
       <c r="S19" s="161"/>
       <c r="T19" s="161"/>
     </row>
     <row r="20" spans="1:20" ht="15.9" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A20" s="338" t="s">
+      <c r="A20" s="349" t="s">
         <v>64</v>
       </c>
-      <c r="B20" s="339"/>
-      <c r="C20" s="339"/>
-      <c r="D20" s="339"/>
+      <c r="B20" s="350"/>
+      <c r="C20" s="350"/>
+      <c r="D20" s="350"/>
       <c r="E20" s="70" t="s">
         <v>0</v>
       </c>
@@ -5198,19 +5199,19 @@
     </row>
     <row r="25" spans="1:20" ht="16.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A25" s="74"/>
-      <c r="B25" s="347" t="s">
+      <c r="B25" s="327" t="s">
         <v>81</v>
       </c>
-      <c r="C25" s="348"/>
-      <c r="D25" s="348"/>
-      <c r="E25" s="348"/>
-      <c r="F25" s="348"/>
-      <c r="G25" s="348"/>
-      <c r="H25" s="348"/>
-      <c r="I25" s="348"/>
-      <c r="J25" s="349"/>
-      <c r="K25" s="344"/>
-      <c r="L25" s="344"/>
+      <c r="C25" s="328"/>
+      <c r="D25" s="328"/>
+      <c r="E25" s="328"/>
+      <c r="F25" s="328"/>
+      <c r="G25" s="328"/>
+      <c r="H25" s="328"/>
+      <c r="I25" s="328"/>
+      <c r="J25" s="329"/>
+      <c r="K25" s="324"/>
+      <c r="L25" s="324"/>
       <c r="M25" s="75"/>
       <c r="N25" s="111"/>
       <c r="O25" s="64"/>
@@ -5241,18 +5242,18 @@
       <c r="H26" s="34" t="s">
         <v>25</v>
       </c>
-      <c r="I26" s="345">
+      <c r="I26" s="325">
         <f>+'DATOS SUELO'!I6</f>
         <v>0</v>
       </c>
-      <c r="J26" s="346"/>
+      <c r="J26" s="326"/>
       <c r="K26" s="79"/>
       <c r="L26" s="35"/>
       <c r="M26" s="80"/>
       <c r="N26" s="111"/>
       <c r="O26" s="65"/>
       <c r="P26" s="66"/>
-      <c r="Q26" s="321" t="s">
+      <c r="Q26" s="332" t="s">
         <v>40</v>
       </c>
       <c r="R26" s="96" t="s">
@@ -5261,7 +5262,7 @@
       <c r="S26" s="96" t="s">
         <v>42</v>
       </c>
-      <c r="T26" s="321" t="s">
+      <c r="T26" s="332" t="s">
         <v>43</v>
       </c>
     </row>
@@ -5278,25 +5279,25 @@
       <c r="H27" s="39" t="s">
         <v>27</v>
       </c>
-      <c r="I27" s="334">
+      <c r="I27" s="345">
         <f>+'DATOS SUELO'!I7</f>
         <v>0</v>
       </c>
-      <c r="J27" s="335"/>
+      <c r="J27" s="346"/>
       <c r="K27" s="79"/>
       <c r="L27" s="35"/>
       <c r="M27" s="80"/>
       <c r="N27" s="111"/>
       <c r="O27" s="65"/>
       <c r="P27" s="66"/>
-      <c r="Q27" s="322"/>
+      <c r="Q27" s="333"/>
       <c r="R27" s="96" t="s">
         <v>44</v>
       </c>
       <c r="S27" s="96" t="s">
         <v>45</v>
       </c>
-      <c r="T27" s="322"/>
+      <c r="T27" s="333"/>
     </row>
     <row r="28" spans="1:20" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A28" s="116"/>
@@ -5311,25 +5312,25 @@
       <c r="H28" s="39" t="s">
         <v>25</v>
       </c>
-      <c r="I28" s="336">
+      <c r="I28" s="347">
         <f>+'DATOS SUELO'!I8</f>
         <v>0</v>
       </c>
-      <c r="J28" s="337"/>
+      <c r="J28" s="348"/>
       <c r="K28" s="40"/>
       <c r="L28" s="41"/>
       <c r="M28" s="81"/>
       <c r="N28" s="119"/>
       <c r="O28" s="65"/>
       <c r="P28" s="66"/>
-      <c r="Q28" s="322"/>
+      <c r="Q28" s="333"/>
       <c r="R28" s="96" t="s">
         <v>46</v>
       </c>
       <c r="S28" s="96" t="s">
         <v>47</v>
       </c>
-      <c r="T28" s="322"/>
+      <c r="T28" s="333"/>
     </row>
     <row r="29" spans="1:20" ht="18.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A29" s="116"/>
@@ -5358,14 +5359,14 @@
       <c r="N29" s="111"/>
       <c r="O29" s="111"/>
       <c r="P29" s="111"/>
-      <c r="Q29" s="323"/>
+      <c r="Q29" s="334"/>
       <c r="R29" s="97" t="s">
         <v>48</v>
       </c>
       <c r="S29" s="97" t="s">
         <v>49</v>
       </c>
-      <c r="T29" s="323"/>
+      <c r="T29" s="334"/>
     </row>
     <row r="30" spans="1:20" ht="18.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A30" s="116"/>
@@ -5619,21 +5620,21 @@
       <c r="P38" s="111"/>
     </row>
     <row r="39" spans="1:20" ht="28.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A39" s="341" t="s">
+      <c r="A39" s="321" t="s">
         <v>84</v>
       </c>
-      <c r="B39" s="341"/>
-      <c r="C39" s="341"/>
-      <c r="D39" s="341"/>
-      <c r="E39" s="341"/>
-      <c r="F39" s="341"/>
-      <c r="G39" s="341"/>
-      <c r="H39" s="341"/>
-      <c r="I39" s="341"/>
-      <c r="J39" s="341"/>
-      <c r="K39" s="341"/>
-      <c r="L39" s="341"/>
-      <c r="M39" s="341"/>
+      <c r="B39" s="321"/>
+      <c r="C39" s="321"/>
+      <c r="D39" s="321"/>
+      <c r="E39" s="321"/>
+      <c r="F39" s="321"/>
+      <c r="G39" s="321"/>
+      <c r="H39" s="321"/>
+      <c r="I39" s="321"/>
+      <c r="J39" s="321"/>
+      <c r="K39" s="321"/>
+      <c r="L39" s="321"/>
+      <c r="M39" s="321"/>
       <c r="N39" s="111"/>
       <c r="O39" s="111"/>
       <c r="P39" s="111"/>
@@ -5870,14 +5871,6 @@
     <protectedRange sqref="F12" name="Rango3_3_1_1_1_1_1_2_1_1_1"/>
   </protectedRanges>
   <mergeCells count="19">
-    <mergeCell ref="A39:M39"/>
-    <mergeCell ref="A8:M8"/>
-    <mergeCell ref="A9:M9"/>
-    <mergeCell ref="K25:L25"/>
-    <mergeCell ref="I26:J26"/>
-    <mergeCell ref="B25:J25"/>
-    <mergeCell ref="C12:J12"/>
-    <mergeCell ref="C11:J11"/>
     <mergeCell ref="T26:T29"/>
     <mergeCell ref="S13:T13"/>
     <mergeCell ref="A16:M16"/>
@@ -5889,6 +5882,14 @@
     <mergeCell ref="A20:D20"/>
     <mergeCell ref="C14:K14"/>
     <mergeCell ref="C13:J13"/>
+    <mergeCell ref="A39:M39"/>
+    <mergeCell ref="A8:M8"/>
+    <mergeCell ref="A9:M9"/>
+    <mergeCell ref="K25:L25"/>
+    <mergeCell ref="I26:J26"/>
+    <mergeCell ref="B25:J25"/>
+    <mergeCell ref="C12:J12"/>
+    <mergeCell ref="C11:J11"/>
   </mergeCells>
   <printOptions horizontalCentered="1"/>
   <pageMargins left="0" right="0" top="0.19685039370078741" bottom="0" header="0.11811023622047245" footer="0"/>
@@ -5941,41 +5942,41 @@
       <c r="P1" s="176"/>
     </row>
     <row r="2" spans="1:16" ht="30" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A2" s="325" t="s">
+      <c r="A2" s="336" t="s">
         <v>80</v>
       </c>
-      <c r="B2" s="326"/>
-      <c r="C2" s="326"/>
-      <c r="D2" s="326"/>
-      <c r="E2" s="326"/>
-      <c r="F2" s="326"/>
-      <c r="G2" s="326"/>
-      <c r="H2" s="326"/>
-      <c r="I2" s="326"/>
-      <c r="J2" s="326"/>
-      <c r="K2" s="326"/>
-      <c r="L2" s="326"/>
-      <c r="M2" s="327"/>
+      <c r="B2" s="337"/>
+      <c r="C2" s="337"/>
+      <c r="D2" s="337"/>
+      <c r="E2" s="337"/>
+      <c r="F2" s="337"/>
+      <c r="G2" s="337"/>
+      <c r="H2" s="337"/>
+      <c r="I2" s="337"/>
+      <c r="J2" s="337"/>
+      <c r="K2" s="337"/>
+      <c r="L2" s="337"/>
+      <c r="M2" s="338"/>
       <c r="N2" s="176"/>
       <c r="O2" s="176"/>
       <c r="P2" s="176"/>
     </row>
     <row r="3" spans="1:16" ht="18" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A3" s="331" t="s">
+      <c r="A3" s="342" t="s">
         <v>23</v>
       </c>
-      <c r="B3" s="332"/>
-      <c r="C3" s="332"/>
-      <c r="D3" s="332"/>
-      <c r="E3" s="332"/>
-      <c r="F3" s="332"/>
-      <c r="G3" s="332"/>
-      <c r="H3" s="332"/>
-      <c r="I3" s="332"/>
-      <c r="J3" s="332"/>
-      <c r="K3" s="332"/>
-      <c r="L3" s="332"/>
-      <c r="M3" s="333"/>
+      <c r="B3" s="343"/>
+      <c r="C3" s="343"/>
+      <c r="D3" s="343"/>
+      <c r="E3" s="343"/>
+      <c r="F3" s="343"/>
+      <c r="G3" s="343"/>
+      <c r="H3" s="343"/>
+      <c r="I3" s="343"/>
+      <c r="J3" s="343"/>
+      <c r="K3" s="343"/>
+      <c r="L3" s="343"/>
+      <c r="M3" s="344"/>
       <c r="N3" s="176"/>
       <c r="O3" s="176"/>
       <c r="P3" s="176"/>
@@ -5999,19 +6000,19 @@
     </row>
     <row r="5" spans="1:16" ht="16.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A5" s="74"/>
-      <c r="B5" s="347" t="s">
+      <c r="B5" s="327" t="s">
         <v>81</v>
       </c>
-      <c r="C5" s="348"/>
-      <c r="D5" s="348"/>
-      <c r="E5" s="348"/>
-      <c r="F5" s="348"/>
-      <c r="G5" s="348"/>
-      <c r="H5" s="348"/>
-      <c r="I5" s="348"/>
-      <c r="J5" s="349"/>
-      <c r="K5" s="344"/>
-      <c r="L5" s="344"/>
+      <c r="C5" s="328"/>
+      <c r="D5" s="328"/>
+      <c r="E5" s="328"/>
+      <c r="F5" s="328"/>
+      <c r="G5" s="328"/>
+      <c r="H5" s="328"/>
+      <c r="I5" s="328"/>
+      <c r="J5" s="329"/>
+      <c r="K5" s="324"/>
+      <c r="L5" s="324"/>
       <c r="M5" s="75"/>
       <c r="N5" s="176"/>
       <c r="O5" s="181"/>
@@ -6383,32 +6384,32 @@
       <c r="J7" s="15"/>
     </row>
     <row r="8" spans="1:13" ht="15.9" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A8" s="342" t="s">
+      <c r="A8" s="322" t="s">
         <v>17</v>
       </c>
-      <c r="B8" s="342"/>
-      <c r="C8" s="342"/>
-      <c r="D8" s="342"/>
-      <c r="E8" s="342"/>
-      <c r="F8" s="342"/>
-      <c r="G8" s="342"/>
-      <c r="H8" s="342"/>
-      <c r="I8" s="342"/>
-      <c r="J8" s="342"/>
+      <c r="B8" s="322"/>
+      <c r="C8" s="322"/>
+      <c r="D8" s="322"/>
+      <c r="E8" s="322"/>
+      <c r="F8" s="322"/>
+      <c r="G8" s="322"/>
+      <c r="H8" s="322"/>
+      <c r="I8" s="322"/>
+      <c r="J8" s="322"/>
     </row>
     <row r="9" spans="1:13" ht="15.9" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A9" s="343">
+      <c r="A9" s="323">
         <v>1</v>
       </c>
-      <c r="B9" s="343"/>
-      <c r="C9" s="343"/>
-      <c r="D9" s="343"/>
-      <c r="E9" s="343"/>
-      <c r="F9" s="343"/>
-      <c r="G9" s="343"/>
-      <c r="H9" s="343"/>
-      <c r="I9" s="343"/>
-      <c r="J9" s="343"/>
+      <c r="B9" s="323"/>
+      <c r="C9" s="323"/>
+      <c r="D9" s="323"/>
+      <c r="E9" s="323"/>
+      <c r="F9" s="323"/>
+      <c r="G9" s="323"/>
+      <c r="H9" s="323"/>
+      <c r="I9" s="323"/>
+      <c r="J9" s="323"/>
       <c r="K9" s="172"/>
       <c r="L9" s="172"/>
       <c r="M9" s="172"/>
@@ -6551,35 +6552,35 @@
       <c r="M15" s="144"/>
     </row>
     <row r="16" spans="1:13" ht="29.4" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A16" s="293" t="s">
+      <c r="A16" s="304" t="s">
         <v>58</v>
       </c>
-      <c r="B16" s="294"/>
-      <c r="C16" s="294"/>
-      <c r="D16" s="294"/>
-      <c r="E16" s="294"/>
-      <c r="F16" s="294"/>
-      <c r="G16" s="294"/>
-      <c r="H16" s="294"/>
-      <c r="I16" s="294"/>
-      <c r="J16" s="295"/>
+      <c r="B16" s="305"/>
+      <c r="C16" s="305"/>
+      <c r="D16" s="305"/>
+      <c r="E16" s="305"/>
+      <c r="F16" s="305"/>
+      <c r="G16" s="305"/>
+      <c r="H16" s="305"/>
+      <c r="I16" s="305"/>
+      <c r="J16" s="306"/>
       <c r="K16" s="144"/>
       <c r="L16" s="144"/>
       <c r="M16" s="144"/>
     </row>
     <row r="17" spans="1:13" ht="18" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A17" s="296" t="s">
+      <c r="A17" s="307" t="s">
         <v>23</v>
       </c>
-      <c r="B17" s="297"/>
-      <c r="C17" s="297"/>
-      <c r="D17" s="297"/>
-      <c r="E17" s="297"/>
-      <c r="F17" s="297"/>
-      <c r="G17" s="297"/>
-      <c r="H17" s="297"/>
-      <c r="I17" s="297"/>
-      <c r="J17" s="298"/>
+      <c r="B17" s="308"/>
+      <c r="C17" s="308"/>
+      <c r="D17" s="308"/>
+      <c r="E17" s="308"/>
+      <c r="F17" s="308"/>
+      <c r="G17" s="308"/>
+      <c r="H17" s="308"/>
+      <c r="I17" s="308"/>
+      <c r="J17" s="309"/>
       <c r="K17" s="144"/>
       <c r="L17" s="144"/>
       <c r="M17" s="144"/>
@@ -6600,18 +6601,18 @@
       <c r="M18" s="144"/>
     </row>
     <row r="19" spans="1:13" ht="15.9" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A19" s="328" t="s">
+      <c r="A19" s="339" t="s">
         <v>20</v>
       </c>
-      <c r="B19" s="329"/>
-      <c r="C19" s="329"/>
-      <c r="D19" s="329"/>
-      <c r="E19" s="329"/>
-      <c r="F19" s="329"/>
-      <c r="G19" s="329"/>
-      <c r="H19" s="329"/>
-      <c r="I19" s="329"/>
-      <c r="J19" s="330"/>
+      <c r="B19" s="340"/>
+      <c r="C19" s="340"/>
+      <c r="D19" s="340"/>
+      <c r="E19" s="340"/>
+      <c r="F19" s="340"/>
+      <c r="G19" s="340"/>
+      <c r="H19" s="340"/>
+      <c r="I19" s="340"/>
+      <c r="J19" s="341"/>
       <c r="L19" s="144"/>
       <c r="M19" s="144"/>
     </row>
@@ -6721,14 +6722,14 @@
     </row>
     <row r="24" spans="1:13" ht="24.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A24" s="49"/>
-      <c r="B24" s="344"/>
-      <c r="C24" s="344"/>
+      <c r="B24" s="324"/>
+      <c r="C24" s="324"/>
       <c r="D24" s="50"/>
       <c r="E24" s="50"/>
       <c r="F24" s="50"/>
       <c r="G24" s="50"/>
-      <c r="H24" s="344"/>
-      <c r="I24" s="344"/>
+      <c r="H24" s="324"/>
+      <c r="I24" s="324"/>
       <c r="J24" s="51"/>
       <c r="K24" s="144"/>
       <c r="L24" s="31"/>
@@ -6940,18 +6941,18 @@
       <c r="M34" s="78"/>
     </row>
     <row r="35" spans="1:13" ht="25.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A35" s="341" t="s">
+      <c r="A35" s="321" t="s">
         <v>84</v>
       </c>
-      <c r="B35" s="341"/>
-      <c r="C35" s="341"/>
-      <c r="D35" s="341"/>
-      <c r="E35" s="341"/>
-      <c r="F35" s="341"/>
-      <c r="G35" s="341"/>
-      <c r="H35" s="341"/>
-      <c r="I35" s="341"/>
-      <c r="J35" s="341"/>
+      <c r="B35" s="321"/>
+      <c r="C35" s="321"/>
+      <c r="D35" s="321"/>
+      <c r="E35" s="321"/>
+      <c r="F35" s="321"/>
+      <c r="G35" s="321"/>
+      <c r="H35" s="321"/>
+      <c r="I35" s="321"/>
+      <c r="J35" s="321"/>
       <c r="K35" s="108"/>
       <c r="L35" s="108"/>
       <c r="M35" s="108"/>
@@ -7197,49 +7198,49 @@
       <c r="M1" s="176"/>
     </row>
     <row r="2" spans="1:13" ht="29.4" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A2" s="325" t="s">
+      <c r="A2" s="336" t="s">
         <v>58</v>
       </c>
-      <c r="B2" s="326"/>
-      <c r="C2" s="326"/>
-      <c r="D2" s="326"/>
-      <c r="E2" s="326"/>
-      <c r="F2" s="326"/>
-      <c r="G2" s="326"/>
-      <c r="H2" s="326"/>
-      <c r="I2" s="326"/>
-      <c r="J2" s="327"/>
+      <c r="B2" s="337"/>
+      <c r="C2" s="337"/>
+      <c r="D2" s="337"/>
+      <c r="E2" s="337"/>
+      <c r="F2" s="337"/>
+      <c r="G2" s="337"/>
+      <c r="H2" s="337"/>
+      <c r="I2" s="337"/>
+      <c r="J2" s="338"/>
       <c r="K2" s="176"/>
       <c r="L2" s="176"/>
       <c r="M2" s="176"/>
     </row>
     <row r="3" spans="1:13" ht="18" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A3" s="331" t="s">
+      <c r="A3" s="342" t="s">
         <v>23</v>
       </c>
-      <c r="B3" s="332"/>
-      <c r="C3" s="332"/>
-      <c r="D3" s="332"/>
-      <c r="E3" s="332"/>
-      <c r="F3" s="332"/>
-      <c r="G3" s="332"/>
-      <c r="H3" s="332"/>
-      <c r="I3" s="332"/>
-      <c r="J3" s="333"/>
+      <c r="B3" s="343"/>
+      <c r="C3" s="343"/>
+      <c r="D3" s="343"/>
+      <c r="E3" s="343"/>
+      <c r="F3" s="343"/>
+      <c r="G3" s="343"/>
+      <c r="H3" s="343"/>
+      <c r="I3" s="343"/>
+      <c r="J3" s="344"/>
       <c r="K3" s="176"/>
       <c r="L3" s="176"/>
       <c r="M3" s="176"/>
     </row>
     <row r="4" spans="1:13" ht="24.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A4" s="49"/>
-      <c r="B4" s="344"/>
-      <c r="C4" s="344"/>
+      <c r="B4" s="324"/>
+      <c r="C4" s="324"/>
       <c r="D4" s="50"/>
       <c r="E4" s="50"/>
       <c r="F4" s="50"/>
       <c r="G4" s="50"/>
-      <c r="H4" s="344"/>
-      <c r="I4" s="344"/>
+      <c r="H4" s="324"/>
+      <c r="I4" s="324"/>
       <c r="J4" s="51"/>
       <c r="K4" s="176"/>
       <c r="L4" s="181"/>

</xml_diff>